<commit_message>
Update Cover Matrix & Defect Report
</commit_message>
<xml_diff>
--- a/Docs/Defect Report.xlsx
+++ b/Docs/Defect Report.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\AtlasLogix-QA-Assessment\Docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Testing\AtlasLogix\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72A4B6CF-330F-4A8F-8724-593E7002EF84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A73612E-C95B-4E9F-BB42-6F0E96781FB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="64">
   <si>
     <t>Defect ID</t>
   </si>
@@ -206,6 +206,45 @@
   </si>
   <si>
     <t>Keyboard focus moves outside the Shipment Details drawer and continues through interactive elements in the underlying Shipments page.</t>
+  </si>
+  <si>
+    <t>DEF-07</t>
+  </si>
+  <si>
+    <t>Tenant name not updated automatically in tenant siwtcher.</t>
+  </si>
+  <si>
+    <t>1- Open Website: https://assessment.nexus-grid.ai/qa/
+2- Log in as the Tenant Administrator.                                 3-Primary Tenant is selected.</t>
+  </si>
+  <si>
+    <t>1- Navigate to the administration page.
+2- Edit primary tenant name.
+3- check the updated name in the tenant switcher.</t>
+  </si>
+  <si>
+    <t>Tenant name still display old name even after refresh the page , the name updated after sign out and sign in again.</t>
+  </si>
+  <si>
+    <t>Tenant new name should be display in the tenant switcher.</t>
+  </si>
+  <si>
+    <t>DEF-08</t>
+  </si>
+  <si>
+    <t>Error message display when try to Change/Activate user role from API</t>
+  </si>
+  <si>
+    <t>1- Open {{baseUrl}}/api/v1/tenants/{{tenantId}}/users/{{targetUserId}}.                                 2-Send the request.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1- Open API collection       2- Log in as the Tenant Administrator.    </t>
+  </si>
+  <si>
+    <t>Role should be updated.</t>
+  </si>
+  <si>
+    <t>Error message display with status code "400"</t>
   </si>
 </sst>
 </file>
@@ -588,7 +627,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J13"/>
+  <dimension ref="A1:J17"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.6640625" style="2" bestFit="1" customWidth="1"/>
@@ -872,14 +911,96 @@
       <c r="H13" s="7"/>
       <c r="I13" s="7"/>
     </row>
+    <row r="14" spans="1:9" ht="129.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="F14" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="G14" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="H14" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I14" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A15" s="7"/>
+      <c r="B15" s="7"/>
+      <c r="C15" s="7"/>
+      <c r="D15" s="7"/>
+      <c r="E15" s="7"/>
+      <c r="F15" s="7"/>
+      <c r="G15" s="7"/>
+      <c r="H15" s="7"/>
+      <c r="I15" s="7"/>
+    </row>
+    <row r="16" spans="1:9" ht="129.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="F16" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="G16" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="H16" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I16" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A17" s="7"/>
+      <c r="B17" s="7"/>
+      <c r="C17" s="7"/>
+      <c r="D17" s="7"/>
+      <c r="E17" s="7"/>
+      <c r="F17" s="7"/>
+      <c r="G17" s="7"/>
+      <c r="H17" s="7"/>
+      <c r="I17" s="7"/>
+    </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="8">
+    <mergeCell ref="A13:I13"/>
+    <mergeCell ref="A15:I15"/>
+    <mergeCell ref="A17:I17"/>
     <mergeCell ref="A3:I3"/>
     <mergeCell ref="A5:I5"/>
     <mergeCell ref="A7:I7"/>
     <mergeCell ref="A9:I9"/>
     <mergeCell ref="A11:I11"/>
-    <mergeCell ref="A13:I13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>